<commit_message>
[ADD] sprint backlog with all the details - last version of the sprint backlog with all the time updated
</commit_message>
<xml_diff>
--- a/documentation/Sprint Backlog Burndown.xlsx
+++ b/documentation/Sprint Backlog Burndown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30602"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\will\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F913FAEB-25AD-4E13-9401-B45FA9B8EED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2450977F-9526-40C0-9267-F6475DE882A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -131,7 +131,7 @@
     <t>Automaticly open &amp; pre-fill the add film or series modals</t>
   </si>
   <si>
-    <t>Delete it from the whish list</t>
+    <t>Delete it from the whish list if mark as watched</t>
   </si>
   <si>
     <t>Estimate Totals</t>
@@ -340,10 +340,10 @@
                   <c:v>15.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.25</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>4.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1444,7 +1444,7 @@
         <v>0.75</v>
       </c>
       <c r="D3" s="2">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -1460,7 +1460,9 @@
       <c r="C4" s="1">
         <v>3</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1473,7 +1475,9 @@
       <c r="C5" s="1">
         <v>1</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1488,7 +1492,9 @@
       <c r="C6" s="1">
         <v>1</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1501,7 +1507,9 @@
       <c r="C7" s="1">
         <v>0.5</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1516,7 +1524,9 @@
       <c r="C8" s="1">
         <v>1.5</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1529,8 +1539,12 @@
       <c r="C9" s="1">
         <v>0.5</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="D9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
@@ -1544,8 +1558,12 @@
       <c r="C10" s="1">
         <v>0.5</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="D10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
@@ -1557,8 +1575,12 @@
       <c r="C11" s="1">
         <v>0.75</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="D11" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
@@ -1570,8 +1592,12 @@
       <c r="C12" s="1">
         <v>0.5</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="D12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
@@ -1585,8 +1611,12 @@
       <c r="C13" s="1">
         <v>0.5</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="D13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
@@ -1598,8 +1628,12 @@
       <c r="C14" s="1">
         <v>0.5</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="D14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
@@ -1611,8 +1645,12 @@
       <c r="C15" s="1">
         <v>0.5</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="D15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
@@ -1626,9 +1664,15 @@
       <c r="C16" s="1">
         <v>1</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7">
@@ -1639,9 +1683,15 @@
       <c r="C17" s="1">
         <v>1</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7">
@@ -1654,9 +1704,15 @@
       <c r="C18" s="1">
         <v>0.5</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="D18" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7">
@@ -1667,9 +1723,15 @@
       <c r="C19" s="1">
         <v>1</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7">
@@ -1680,9 +1742,15 @@
       <c r="C20" s="1">
         <v>0.75</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="D20" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
       <c r="G20" s="2"/>
     </row>
     <row r="21" spans="1:7">
@@ -1803,11 +1871,11 @@
       </c>
       <c r="D33" s="3">
         <f t="shared" ref="D33:G33" si="0">SUM(D3:D32)</f>
-        <v>1.25</v>
+        <v>8</v>
       </c>
       <c r="E33" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F33" s="3">
         <f t="shared" si="0"/>

</xml_diff>